<commit_message>
text mining test on 10 companies
</commit_message>
<xml_diff>
--- a/Data/data_TextMining/df_Pfizer_reference.xlsx
+++ b/Data/data_TextMining/df_Pfizer_reference.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P49"/>
+  <dimension ref="A1:Q49"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -387,50 +387,55 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
+          <t>yr</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
           <t>n_statement</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>goal_desc</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>ind</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Industry</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>ind_agg</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>ind_7sys</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>ind_3</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>Region</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Continent</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>ns</t>
         </is>
@@ -454,12 +459,12 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>1.1</t>
+          <t>1_g</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>g</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
@@ -468,41 +473,39 @@
         </is>
       </c>
       <c r="G2">
+        <v>2018</v>
+      </c>
+      <c r="H2">
         <v>1</v>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>No Poverty</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Healthcare and life sciences</t>
-        </is>
-      </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O2" t="inlineStr">
@@ -511,6 +514,11 @@
         </is>
       </c>
       <c r="P2" t="inlineStr">
+        <is>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
         <is>
           <t>[1,2)</t>
         </is>
@@ -529,60 +537,58 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>10</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>10_3</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>3.4</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>SDG3</t>
+          <t>SDG10</t>
         </is>
       </c>
       <c r="G3">
-        <v>1382</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>Good Health And Well-Being</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H3">
+        <v>1</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Reduced Inequalities</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
@@ -592,7 +598,12 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>[40,1.38e+03]</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>[1,2)</t>
         </is>
       </c>
     </row>
@@ -609,60 +620,58 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>11</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>3.2</t>
+          <t>11_g</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>g</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>SDG3</t>
+          <t>SDG11</t>
         </is>
       </c>
       <c r="G4">
-        <v>80</v>
-      </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Good Health And Well-Being</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H4">
+        <v>32</v>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Sustainable Cities And Communities</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N4" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
@@ -672,7 +681,12 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>[40,1.38e+03]</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>[18,37)</t>
         </is>
       </c>
     </row>
@@ -689,60 +703,58 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>12</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>12_2</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>SDG3</t>
+          <t>SDG12</t>
         </is>
       </c>
       <c r="G5">
-        <v>8</v>
-      </c>
-      <c r="H5" t="inlineStr">
-        <is>
-          <t>Good Health And Well-Being</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H5">
+        <v>7</v>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Responsible Consumption And Production</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M5" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N5" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
@@ -752,7 +764,12 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>[7,12)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>[7,11)</t>
         </is>
       </c>
     </row>
@@ -769,60 +786,58 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>12</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>12_4</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>SDG3</t>
+          <t>SDG12</t>
         </is>
       </c>
       <c r="G6">
-        <v>10</v>
-      </c>
-      <c r="H6" t="inlineStr">
-        <is>
-          <t>Good Health And Well-Being</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H6">
+        <v>75</v>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Responsible Consumption And Production</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -832,7 +847,12 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>[7,12)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>[37,1.38e+03]</t>
         </is>
       </c>
     </row>
@@ -849,60 +869,58 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>12</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>3.c</t>
+          <t>12_5</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>c</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>SDG3</t>
+          <t>SDG12</t>
         </is>
       </c>
       <c r="G7">
-        <v>157</v>
-      </c>
-      <c r="H7" t="inlineStr">
-        <is>
-          <t>Good Health And Well-Being</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Responsible Consumption And Production</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
@@ -912,7 +930,12 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>[40,1.38e+03]</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>[1,2)</t>
         </is>
       </c>
     </row>
@@ -929,60 +952,58 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>12</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>3.a</t>
+          <t>12_g</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>g</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>SDG3</t>
+          <t>SDG12</t>
         </is>
       </c>
       <c r="G8">
-        <v>39</v>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>Good Health And Well-Being</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H8">
+        <v>47</v>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Responsible Consumption And Production</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L8" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M8" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N8" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
@@ -992,7 +1013,12 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>[20,40)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>[37,1.38e+03]</t>
         </is>
       </c>
     </row>
@@ -1009,60 +1035,58 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>13</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>3.5</t>
+          <t>13_2</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>SDG3</t>
+          <t>SDG13</t>
         </is>
       </c>
       <c r="G9">
-        <v>36</v>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Good Health And Well-Being</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H9">
+        <v>25</v>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Climate Action</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M9" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N9" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
@@ -1072,7 +1096,12 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>[20,40)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>[18,37)</t>
         </is>
       </c>
     </row>
@@ -1089,60 +1118,58 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>13</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>13_a</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>a</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>SDG3</t>
+          <t>SDG13</t>
         </is>
       </c>
       <c r="G10">
-        <v>3</v>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>Good Health And Well-Being</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H10">
+        <v>33</v>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Climate Action</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M10" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N10" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
@@ -1152,7 +1179,12 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>[3,5)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>[18,37)</t>
         </is>
       </c>
     </row>
@@ -1169,60 +1201,58 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>16</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>3.3</t>
+          <t>16_6</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>SDG3</t>
+          <t>SDG16</t>
         </is>
       </c>
       <c r="G11">
+        <v>2018</v>
+      </c>
+      <c r="H11">
         <v>1</v>
       </c>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>Good Health And Well-Being</t>
-        </is>
-      </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Peace, Justice And Strong Institutions</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
@@ -1231,6 +1261,11 @@
         </is>
       </c>
       <c r="P11" t="inlineStr">
+        <is>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
         <is>
           <t>[1,2)</t>
         </is>
@@ -1249,60 +1284,58 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>16</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>3.9</t>
+          <t>16_g</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>g</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>SDG3</t>
+          <t>SDG16</t>
         </is>
       </c>
       <c r="G12">
-        <v>7</v>
-      </c>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>Good Health And Well-Being</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H12">
+        <v>10</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Peace, Justice And Strong Institutions</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
@@ -1312,7 +1345,12 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>[7,12)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>[7,11)</t>
         </is>
       </c>
     </row>
@@ -1329,60 +1367,58 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>17</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>3.b</t>
+          <t>17_16</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>16</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>SDG3</t>
+          <t>SDG17</t>
         </is>
       </c>
       <c r="G13">
-        <v>38</v>
-      </c>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>Good Health And Well-Being</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H13">
+        <v>71</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Partnersip for Goals</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
@@ -1392,7 +1428,12 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>[20,40)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>[37,1.38e+03]</t>
         </is>
       </c>
     </row>
@@ -1409,60 +1450,58 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>17</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>3.4</t>
+          <t>17_16</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>16</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>SDG3</t>
+          <t>SDG17</t>
         </is>
       </c>
       <c r="G14">
-        <v>11</v>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>Good Health And Well-Being</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H14">
+        <v>4</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Partnersip for Goals</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
@@ -1472,7 +1511,12 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>[7,12)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>[4,7)</t>
         </is>
       </c>
     </row>
@@ -1489,60 +1533,58 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>17</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>3.7</t>
+          <t>17_9</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>9</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>SDG3</t>
+          <t>SDG17</t>
         </is>
       </c>
       <c r="G15">
-        <v>33</v>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>Good Health And Well-Being</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H15">
+        <v>2</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Partnersip for Goals</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
@@ -1552,7 +1594,12 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>[20,40)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>[2,3)</t>
         </is>
       </c>
     </row>
@@ -1574,12 +1621,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>3.7</t>
+          <t>3_1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
@@ -1588,41 +1635,39 @@
         </is>
       </c>
       <c r="G16">
-        <v>46</v>
-      </c>
-      <c r="H16" t="inlineStr">
+        <v>2018</v>
+      </c>
+      <c r="H16">
+        <v>24</v>
+      </c>
+      <c r="I16" t="inlineStr">
         <is>
           <t>Good Health And Well-Being</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>Healthcare and life sciences</t>
-        </is>
-      </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M16" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N16" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
@@ -1632,7 +1677,12 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>[40,1.38e+03]</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>[18,37)</t>
         </is>
       </c>
     </row>
@@ -1654,12 +1704,12 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>3.1</t>
+          <t>3_2</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -1668,41 +1718,39 @@
         </is>
       </c>
       <c r="G17">
-        <v>24</v>
-      </c>
-      <c r="H17" t="inlineStr">
+        <v>2018</v>
+      </c>
+      <c r="H17">
+        <v>80</v>
+      </c>
+      <c r="I17" t="inlineStr">
         <is>
           <t>Good Health And Well-Being</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>Healthcare and life sciences</t>
-        </is>
-      </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M17" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N17" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
@@ -1712,7 +1760,12 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>[20,40)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>[37,1.38e+03]</t>
         </is>
       </c>
     </row>
@@ -1729,60 +1782,58 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>4.2</t>
+          <t>3_3</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>SDG4</t>
+          <t>SDG3</t>
         </is>
       </c>
       <c r="G18">
-        <v>5</v>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>Quality Education</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H18">
+        <v>1</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Good Health And Well-Being</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M18" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N18" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
@@ -1792,7 +1843,12 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>[5,7)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>[1,2)</t>
         </is>
       </c>
     </row>
@@ -1809,60 +1865,58 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>5.b</t>
+          <t>3_3</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>SDG5</t>
+          <t>SDG3</t>
         </is>
       </c>
       <c r="G19">
-        <v>6</v>
-      </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>Gender Equality</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H19">
+        <v>10</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Good Health And Well-Being</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
@@ -1872,7 +1926,12 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>[5,7)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>[7,11)</t>
         </is>
       </c>
     </row>
@@ -1889,60 +1948,58 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>3_3</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>SDG5</t>
+          <t>SDG3</t>
         </is>
       </c>
       <c r="G20">
-        <v>2</v>
-      </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>Gender Equality</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H20">
+        <v>8</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Good Health And Well-Being</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K20" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M20" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N20" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
@@ -1952,7 +2009,12 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>[2,3)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr">
+        <is>
+          <t>[7,11)</t>
         </is>
       </c>
     </row>
@@ -1969,60 +2031,58 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>5.5</t>
+          <t>3_4</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>SDG5</t>
+          <t>SDG3</t>
         </is>
       </c>
       <c r="G21">
-        <v>5</v>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>Gender Equality</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H21">
+        <v>11</v>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Good Health And Well-Being</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M21" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N21" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
@@ -2032,7 +2092,12 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>[5,7)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr">
+        <is>
+          <t>[11,18)</t>
         </is>
       </c>
     </row>
@@ -2049,60 +2114,58 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>3_5</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
           <t>5</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>5.a</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>a</t>
-        </is>
-      </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>SDG5</t>
+          <t>SDG3</t>
         </is>
       </c>
       <c r="G22">
-        <v>1</v>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>Gender Equality</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H22">
+        <v>36</v>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Good Health And Well-Being</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M22" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N22" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
@@ -2112,7 +2175,12 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>[1,2)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr">
+        <is>
+          <t>[18,37)</t>
         </is>
       </c>
     </row>
@@ -2129,60 +2197,58 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>3_7</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>SDG5</t>
+          <t>SDG3</t>
         </is>
       </c>
       <c r="G23">
-        <v>20</v>
-      </c>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>Gender Equality</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H23">
+        <v>33</v>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Good Health And Well-Being</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M23" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
@@ -2192,7 +2258,12 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>[20,40)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr">
+        <is>
+          <t>[18,37)</t>
         </is>
       </c>
     </row>
@@ -2209,60 +2280,58 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>5.a</t>
+          <t>3_7</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>7</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>SDG5</t>
+          <t>SDG3</t>
         </is>
       </c>
       <c r="G24">
-        <v>21</v>
-      </c>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>Gender Equality</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H24">
+        <v>46</v>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Good Health And Well-Being</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K24" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M24" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
@@ -2272,7 +2341,12 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>[20,40)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr">
+        <is>
+          <t>[37,1.38e+03]</t>
         </is>
       </c>
     </row>
@@ -2289,60 +2363,58 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>6.3</t>
+          <t>3_9</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>9</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>SDG6</t>
+          <t>SDG3</t>
         </is>
       </c>
       <c r="G25">
-        <v>1</v>
-      </c>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>Clean Water And Sanitation</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H25">
+        <v>3</v>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Good Health And Well-Being</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K25" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M25" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N25" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
@@ -2352,7 +2424,12 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>[1,2)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr">
+        <is>
+          <t>[3,4)</t>
         </is>
       </c>
     </row>
@@ -2369,60 +2446,58 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>6.2</t>
+          <t>3_9</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>SDG6</t>
+          <t>SDG3</t>
         </is>
       </c>
       <c r="G26">
-        <v>13</v>
-      </c>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>Clean Water And Sanitation</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H26">
+        <v>7</v>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Good Health And Well-Being</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M26" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N26" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
@@ -2432,7 +2507,12 @@
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>[12,20)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr">
+        <is>
+          <t>[7,11)</t>
         </is>
       </c>
     </row>
@@ -2449,60 +2529,58 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>6.1</t>
+          <t>3_a</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>a</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>SDG6</t>
+          <t>SDG3</t>
         </is>
       </c>
       <c r="G27">
-        <v>1</v>
-      </c>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>Clean Water And Sanitation</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H27">
+        <v>39</v>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Good Health And Well-Being</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M27" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N27" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
@@ -2512,7 +2590,12 @@
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>[1,2)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr">
+        <is>
+          <t>[37,1.38e+03]</t>
         </is>
       </c>
     </row>
@@ -2529,60 +2612,58 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>6.4</t>
+          <t>3_b</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>b</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>SDG6</t>
+          <t>SDG3</t>
         </is>
       </c>
       <c r="G28">
-        <v>13</v>
-      </c>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>Clean Water And Sanitation</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H28">
+        <v>38</v>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Good Health And Well-Being</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M28" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N28" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
@@ -2592,7 +2673,12 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>[12,20)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr">
+        <is>
+          <t>[37,1.38e+03]</t>
         </is>
       </c>
     </row>
@@ -2609,60 +2695,58 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>7.a</t>
+          <t>3_b</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>b</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>SDG7</t>
+          <t>SDG3</t>
         </is>
       </c>
       <c r="G29">
-        <v>2</v>
-      </c>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>Affordable And Clean Energy</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H29">
+        <v>157</v>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Good Health And Well-Being</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K29" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M29" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N29" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
@@ -2672,7 +2756,12 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>[2,3)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr">
+        <is>
+          <t>[37,1.38e+03]</t>
         </is>
       </c>
     </row>
@@ -2689,60 +2778,58 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>3</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>7.3</t>
+          <t>3_g</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>g</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>SDG7</t>
+          <t>SDG3</t>
         </is>
       </c>
       <c r="G30">
-        <v>5</v>
-      </c>
-      <c r="H30" t="inlineStr">
-        <is>
-          <t>Affordable And Clean Energy</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H30">
+        <v>1382</v>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Good Health And Well-Being</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M30" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N30" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
@@ -2752,7 +2839,12 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>[5,7)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr">
+        <is>
+          <t>[37,1.38e+03]</t>
         </is>
       </c>
     </row>
@@ -2769,60 +2861,58 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>4</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>8.1</t>
+          <t>4_2</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>SDG8</t>
+          <t>SDG4</t>
         </is>
       </c>
       <c r="G31">
-        <v>17</v>
-      </c>
-      <c r="H31" t="inlineStr">
-        <is>
-          <t>Decent Work And Economic Growth</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H31">
+        <v>5</v>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Quality Education</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M31" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N31" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
@@ -2832,7 +2922,12 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>[12,20)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr">
+        <is>
+          <t>[4,7)</t>
         </is>
       </c>
     </row>
@@ -2849,12 +2944,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>5_5</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -2864,45 +2959,43 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>SDG8</t>
+          <t>SDG5</t>
         </is>
       </c>
       <c r="G32">
-        <v>13</v>
-      </c>
-      <c r="H32" t="inlineStr">
-        <is>
-          <t>Decent Work And Economic Growth</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H32">
+        <v>5</v>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Gender Equality</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M32" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N32" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
@@ -2912,7 +3005,12 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>[12,20)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>[4,7)</t>
         </is>
       </c>
     </row>
@@ -2929,60 +3027,58 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>8.5</t>
+          <t>5_6</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>SDG8</t>
+          <t>SDG5</t>
         </is>
       </c>
       <c r="G33">
-        <v>9</v>
-      </c>
-      <c r="H33" t="inlineStr">
-        <is>
-          <t>Decent Work And Economic Growth</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H33">
+        <v>2</v>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Gender Equality</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M33" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N33" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
@@ -2992,7 +3088,12 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>[7,12)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>[2,3)</t>
         </is>
       </c>
     </row>
@@ -3009,60 +3110,58 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>9.b</t>
+          <t>5_6</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>b</t>
+          <t>6</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>SDG9</t>
+          <t>SDG5</t>
         </is>
       </c>
       <c r="G34">
-        <v>7</v>
-      </c>
-      <c r="H34" t="inlineStr">
-        <is>
-          <t>Industry, Innovation And Infrastructure</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H34">
+        <v>20</v>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Gender Equality</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M34" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N34" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
@@ -3072,7 +3171,12 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>[7,12)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>[18,37)</t>
         </is>
       </c>
     </row>
@@ -3089,60 +3193,58 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>9.4</t>
+          <t>5_a</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>a</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>SDG9</t>
+          <t>SDG5</t>
         </is>
       </c>
       <c r="G35">
-        <v>8</v>
-      </c>
-      <c r="H35" t="inlineStr">
-        <is>
-          <t>Industry, Innovation And Infrastructure</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H35">
+        <v>1</v>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Gender Equality</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M35" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N35" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
@@ -3152,7 +3254,12 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>[7,12)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>[1,2)</t>
         </is>
       </c>
     </row>
@@ -3169,60 +3276,58 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>5_b</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>b</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>SDG10</t>
+          <t>SDG5</t>
         </is>
       </c>
       <c r="G36">
-        <v>1</v>
-      </c>
-      <c r="H36" t="inlineStr">
-        <is>
-          <t>Reduced Inequalities</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H36">
+        <v>6</v>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Gender Equality</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N36" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
@@ -3232,7 +3337,12 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>[1,2)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>[4,7)</t>
         </is>
       </c>
     </row>
@@ -3249,60 +3359,58 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>5</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>11.6</t>
+          <t>5_g</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>g</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>SDG11</t>
+          <t>SDG5</t>
         </is>
       </c>
       <c r="G37">
-        <v>32</v>
-      </c>
-      <c r="H37" t="inlineStr">
-        <is>
-          <t>Sustainable Cities And Communities</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H37">
+        <v>21</v>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Gender Equality</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N37" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
@@ -3312,7 +3420,12 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>[20,40)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>[18,37)</t>
         </is>
       </c>
     </row>
@@ -3329,60 +3442,58 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>12.5</t>
+          <t>6_1</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>SDG12</t>
+          <t>SDG6</t>
         </is>
       </c>
       <c r="G38">
+        <v>2018</v>
+      </c>
+      <c r="H38">
         <v>1</v>
       </c>
-      <c r="H38" t="inlineStr">
-        <is>
-          <t>Responsible Consumption And Production</t>
-        </is>
-      </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Clean Water And Sanitation</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N38" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
@@ -3391,6 +3502,11 @@
         </is>
       </c>
       <c r="P38" t="inlineStr">
+        <is>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q38" t="inlineStr">
         <is>
           <t>[1,2)</t>
         </is>
@@ -3409,60 +3525,58 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>12.4</t>
+          <t>6_3</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>SDG12</t>
+          <t>SDG6</t>
         </is>
       </c>
       <c r="G39">
-        <v>75</v>
-      </c>
-      <c r="H39" t="inlineStr">
-        <is>
-          <t>Responsible Consumption And Production</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H39">
+        <v>1</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Clean Water And Sanitation</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M39" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N39" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
@@ -3472,7 +3586,12 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>[40,1.38e+03]</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>[1,2)</t>
         </is>
       </c>
     </row>
@@ -3489,60 +3608,58 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>12.1</t>
+          <t>6_4</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>SDG12</t>
+          <t>SDG6</t>
         </is>
       </c>
       <c r="G40">
-        <v>47</v>
-      </c>
-      <c r="H40" t="inlineStr">
-        <is>
-          <t>Responsible Consumption And Production</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H40">
+        <v>13</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Clean Water And Sanitation</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M40" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N40" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
@@ -3552,7 +3669,12 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>[40,1.38e+03]</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>[11,18)</t>
         </is>
       </c>
     </row>
@@ -3569,60 +3691,58 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>6</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>12.2</t>
+          <t>6_g</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>g</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>SDG12</t>
+          <t>SDG6</t>
         </is>
       </c>
       <c r="G41">
-        <v>7</v>
-      </c>
-      <c r="H41" t="inlineStr">
-        <is>
-          <t>Responsible Consumption And Production</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H41">
+        <v>13</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Clean Water And Sanitation</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M41" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N41" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
@@ -3632,7 +3752,12 @@
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>[7,12)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>[11,18)</t>
         </is>
       </c>
     </row>
@@ -3649,60 +3774,58 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>13.a</t>
+          <t>7_3</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>a</t>
+          <t>3</t>
         </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>SDG13</t>
+          <t>SDG7</t>
         </is>
       </c>
       <c r="G42">
-        <v>33</v>
-      </c>
-      <c r="H42" t="inlineStr">
-        <is>
-          <t>Climate Action</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H42">
+        <v>5</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Affordable And Clean Energy</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M42" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N42" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
@@ -3712,7 +3835,12 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>[20,40)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>[4,7)</t>
         </is>
       </c>
     </row>
@@ -3729,60 +3857,58 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>13</t>
+          <t>7</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>13.2</t>
+          <t>7_g</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>g</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>SDG13</t>
+          <t>SDG7</t>
         </is>
       </c>
       <c r="G43">
-        <v>25</v>
-      </c>
-      <c r="H43" t="inlineStr">
-        <is>
-          <t>Climate Action</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H43">
+        <v>2</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Affordable And Clean Energy</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M43" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N43" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
@@ -3792,7 +3918,12 @@
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>[20,40)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>[2,3)</t>
         </is>
       </c>
     </row>
@@ -3809,60 +3940,58 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>16.3</t>
+          <t>8_5</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>SDG16</t>
+          <t>SDG8</t>
         </is>
       </c>
       <c r="G44">
-        <v>10</v>
-      </c>
-      <c r="H44" t="inlineStr">
-        <is>
-          <t>Peace, Justice And Strong Institutions</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H44">
+        <v>9</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Decent Work And Economic Growth</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M44" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N44" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
@@ -3872,7 +4001,12 @@
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>[7,12)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>[7,11)</t>
         </is>
       </c>
     </row>
@@ -3889,60 +4023,58 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>16.6</t>
+          <t>8_5</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>SDG16</t>
+          <t>SDG8</t>
         </is>
       </c>
       <c r="G45">
-        <v>1</v>
-      </c>
-      <c r="H45" t="inlineStr">
-        <is>
-          <t>Peace, Justice And Strong Institutions</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H45">
+        <v>13</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Decent Work And Economic Growth</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M45" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N45" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
@@ -3952,7 +4084,12 @@
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>[1,2)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>[11,18)</t>
         </is>
       </c>
     </row>
@@ -3969,60 +4106,58 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>8</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>17.9</t>
+          <t>8_g</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>g</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>SDG17</t>
+          <t>SDG8</t>
         </is>
       </c>
       <c r="G46">
-        <v>2</v>
-      </c>
-      <c r="H46" t="inlineStr">
-        <is>
-          <t>Partnersip for Goals</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H46">
+        <v>17</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Decent Work And Economic Growth</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M46" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N46" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
@@ -4032,7 +4167,12 @@
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>[2,3)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>[11,18)</t>
         </is>
       </c>
     </row>
@@ -4049,60 +4189,58 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>17.6</t>
+          <t>9_b</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>b</t>
         </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>SDG17</t>
+          <t>SDG9</t>
         </is>
       </c>
       <c r="G47">
-        <v>4</v>
-      </c>
-      <c r="H47" t="inlineStr">
-        <is>
-          <t>Partnersip for Goals</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H47">
+        <v>7</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Industry, Innovation And Infrastructure</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M47" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N47" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
@@ -4112,7 +4250,12 @@
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>[3,5)</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>[7,11)</t>
         </is>
       </c>
     </row>
@@ -4129,60 +4272,58 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>9</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>17.16</t>
+          <t>9_g</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>g</t>
         </is>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>SDG17</t>
+          <t>SDG9</t>
         </is>
       </c>
       <c r="G48">
-        <v>71</v>
-      </c>
-      <c r="H48" t="inlineStr">
-        <is>
-          <t>Partnersip for Goals</t>
-        </is>
+        <v>2018</v>
+      </c>
+      <c r="H48">
+        <v>8</v>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Industry, Innovation And Infrastructure</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M48" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N48" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
@@ -4192,7 +4333,12 @@
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>[40,1.38e+03]</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>[7,11)</t>
         </is>
       </c>
     </row>
@@ -4217,47 +4363,50 @@
           <t>SDGs</t>
         </is>
       </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>g</t>
+        </is>
+      </c>
       <c r="F49" t="inlineStr">
         <is>
           <t>SDG</t>
         </is>
       </c>
       <c r="G49">
+        <v>2018</v>
+      </c>
+      <c r="H49">
         <v>50</v>
       </c>
-      <c r="H49" t="inlineStr">
+      <c r="I49" t="inlineStr">
         <is>
           <t>in general</t>
         </is>
       </c>
-      <c r="I49" t="inlineStr">
-        <is>
-          <t>Healthcare and life sciences</t>
-        </is>
-      </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>Pharmaceutical industry</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>Health care</t>
+          <t>Pharmaceutical industry</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>Healthcare and life sciences</t>
+          <t>Health care</t>
         </is>
       </c>
       <c r="M49" t="inlineStr">
         <is>
-          <t>Tertiary</t>
+          <t>Healthcare and life sciences</t>
         </is>
       </c>
       <c r="N49" t="inlineStr">
         <is>
-          <t>Americas</t>
+          <t>Tertiary</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
@@ -4267,7 +4416,12 @@
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>[40,1.38e+03]</t>
+          <t>Americas</t>
+        </is>
+      </c>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>[37,1.38e+03]</t>
         </is>
       </c>
     </row>

</xml_diff>